<commit_message>
Project documentation, feature importance calculation & visualization.
</commit_message>
<xml_diff>
--- a/WeeklyPredictions.xlsx
+++ b/WeeklyPredictions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkArea\Workspaces\ProfessionalCourses\AI-ML_CapstoneProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E4A9FF8-3F18-4ADB-81AC-CB1884AAD7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D06F9D-E08C-4026-AAF3-1646E3E5CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="354" yWindow="600" windowWidth="22500" windowHeight="12852" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="354" yWindow="600" windowWidth="22500" windowHeight="12852" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Function 1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Weeks 5, 6, 7
</commit_message>
<xml_diff>
--- a/WeeklyPredictions.xlsx
+++ b/WeeklyPredictions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkArea\Workspaces\ProfessionalCourses\AI-ML_CapstoneProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369F7F80-D2F0-4658-A85A-78463E02E457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B882584D-066F-4F49-A138-B210D507CA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58440" yWindow="600" windowWidth="36765" windowHeight="19575" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="61110" yWindow="825" windowWidth="32415" windowHeight="18675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Function 1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="103">
   <si>
     <t>Input (feature) dimension:</t>
   </si>
@@ -481,6 +481,42 @@
   </si>
   <si>
     <t>[0.070000, 0.046261, 0.100000, 0.100000, 0.047011, 0.047261, 0.047511, 0.047761]</t>
+  </si>
+  <si>
+    <t>[0.794794, 0.795795]</t>
+  </si>
+  <si>
+    <t>[0.512512, 0.513513]</t>
+  </si>
+  <si>
+    <t>[0.450000, 0.500000, 0.500000]</t>
+  </si>
+  <si>
+    <t>Confidence interval/ETA</t>
+  </si>
+  <si>
+    <t>eta = 0.01</t>
+  </si>
+  <si>
+    <t>Matern(length_scale=0.1, length_scale_bounds=(1e-3, 1e3), nu=1.5)</t>
+  </si>
+  <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>[0.360180, 0.360680, 0.361180, 0.361680]</t>
+  </si>
+  <si>
+    <t>[1.000000, 0.400000, 1.000000, 1.000000]</t>
+  </si>
+  <si>
+    <t>[0.420168, 0.420568, 0.420968, 0.700000, 0.060000]</t>
+  </si>
+  <si>
+    <t>[0.366122, 0.366455, 0.366788, 0.367122, 0.367455, 0.680000]</t>
+  </si>
+  <si>
+    <t>[0.015000, 0.190000, 0.000000, 0.000000, 0.190000, 0.190000, 0.190000, 0.190000]</t>
   </si>
 </sst>
 </file>
@@ -744,7 +780,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -875,6 +911,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1179,7 +1233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:N31"/>
+  <dimension ref="B3:N35"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13.3125" customWidth="1"/>
@@ -1736,6 +1790,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="32" spans="2:14">
+      <c r="B32" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="23">
+        <v>6</v>
+      </c>
+      <c r="D32" s="27">
+        <v>0.384384</v>
+      </c>
+      <c r="E32" s="27">
+        <v>0.38538499999999998</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="H32" s="24">
+        <v>6</v>
+      </c>
+      <c r="I32" s="24"/>
+      <c r="J32" s="28">
+        <v>1.54339407934348E-4</v>
+      </c>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24"/>
+      <c r="N32" s="24"/>
+    </row>
+    <row r="33" spans="2:14" ht="43.2">
+      <c r="G33" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="13">
+        <f>MAX(L31,J32)</f>
+        <v>1.54339407934348E-4</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14">
+      <c r="B34" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="23">
+        <v>7</v>
+      </c>
+      <c r="D34" s="27">
+        <v>0.794794</v>
+      </c>
+      <c r="E34" s="27">
+        <v>0.79579500000000003</v>
+      </c>
+      <c r="G34" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="H34" s="24">
+        <v>7</v>
+      </c>
+      <c r="I34" s="24"/>
+      <c r="J34" s="28">
+        <v>3.8815429764520301E-39</v>
+      </c>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
+    </row>
+    <row r="35" spans="2:14">
+      <c r="L35" s="13">
+        <f>MAX(L33,J34)</f>
+        <v>1.54339407934348E-4</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B9:C18"/>
@@ -1752,7 +1886,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{670CB941-049A-4FC0-8F09-1656ED8CE3C7}">
-  <dimension ref="B3:N32"/>
+  <dimension ref="B3:N36"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -2316,6 +2450,84 @@
         <v>1</v>
       </c>
     </row>
+    <row r="33" spans="2:13">
+      <c r="B33" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="23">
+        <v>6</v>
+      </c>
+      <c r="D33" s="27">
+        <v>0.75</v>
+      </c>
+      <c r="E33" s="27">
+        <v>0.9</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="H33" s="24">
+        <v>6</v>
+      </c>
+      <c r="I33" s="24"/>
+      <c r="J33" s="26">
+        <v>0.52262959533611497</v>
+      </c>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+    </row>
+    <row r="34" spans="2:13" ht="43.2">
+      <c r="G34" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="H34" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L34" s="21">
+        <f>MAX(L32,J33)</f>
+        <v>0.70032323557308995</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13">
+      <c r="B35" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="23">
+        <v>7</v>
+      </c>
+      <c r="D35" s="27">
+        <v>0.51251199999999997</v>
+      </c>
+      <c r="E35" s="27">
+        <v>0.513513</v>
+      </c>
+      <c r="G35" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="H35" s="24">
+        <v>7</v>
+      </c>
+      <c r="I35" s="24"/>
+      <c r="J35" s="26">
+        <v>0.61916671697804904</v>
+      </c>
+      <c r="K35" s="24"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="24"/>
+    </row>
+    <row r="36" spans="2:13">
+      <c r="L36" s="21">
+        <f>MAX(L34,J35)</f>
+        <v>0.70032323557308995</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B4:C4"/>
@@ -2332,7 +2544,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31898AF6-32B3-4A29-BBAB-B50A72E3787B}">
-  <dimension ref="B3:O36"/>
+  <dimension ref="B3:O40"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -3033,6 +3245,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="37" spans="2:15">
+      <c r="B37" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="23">
+        <v>6</v>
+      </c>
+      <c r="D37" s="27">
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="E37" s="27">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F37" s="27">
+        <v>0.56599999999999995</v>
+      </c>
+      <c r="H37" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="I37" s="24">
+        <v>6</v>
+      </c>
+      <c r="J37" s="24"/>
+      <c r="K37" s="26">
+        <v>-2.5600644844795201E-2</v>
+      </c>
+      <c r="L37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="N37" s="24"/>
+      <c r="O37" s="24"/>
+    </row>
+    <row r="38" spans="2:15" ht="28.8">
+      <c r="H38" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M38" s="21">
+        <f>MAX(M36,K37)</f>
+        <v>-3.7555388348285302E-3</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="2:15">
+      <c r="B39" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="23">
+        <v>7</v>
+      </c>
+      <c r="D39" s="27">
+        <v>0.45</v>
+      </c>
+      <c r="E39" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="F39" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="H39" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="I39" s="24">
+        <v>7</v>
+      </c>
+      <c r="J39" s="24"/>
+      <c r="K39" s="26">
+        <v>-3.7555388348285302E-3</v>
+      </c>
+      <c r="L39" s="24"/>
+      <c r="M39" s="24"/>
+      <c r="N39" s="24"/>
+      <c r="O39" s="24"/>
+    </row>
+    <row r="40" spans="2:15">
+      <c r="M40" s="21">
+        <f>MAX(M38,K39)</f>
+        <v>-3.7555388348285302E-3</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B9:C23"/>
@@ -3050,7 +3342,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7581826F-7241-48DF-A0E8-08483F533A08}">
-  <dimension ref="B3:P50"/>
+  <dimension ref="B3:P54"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -3111,31 +3403,31 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="21.3">
+    <row r="8" spans="2:16" ht="28.8">
       <c r="B8" s="41"/>
       <c r="C8" s="41"/>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="K8" s="15" t="s">
+      <c r="J8" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="18" t="s">
+      <c r="L8" s="47" t="s">
         <v>10</v>
       </c>
       <c r="M8" s="1"/>
@@ -4145,6 +4437,98 @@
       </c>
       <c r="P50" s="32" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="2:16">
+      <c r="B51" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="23">
+        <v>6</v>
+      </c>
+      <c r="D51" s="27">
+        <v>0.35817900000000003</v>
+      </c>
+      <c r="E51" s="27">
+        <v>0.35867900000000003</v>
+      </c>
+      <c r="F51" s="27">
+        <v>0.35917900000000003</v>
+      </c>
+      <c r="G51" s="27">
+        <v>0.35967900000000003</v>
+      </c>
+      <c r="I51" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="J51" s="24">
+        <v>6</v>
+      </c>
+      <c r="K51" s="24"/>
+      <c r="L51" s="26">
+        <v>0.73775846532035805</v>
+      </c>
+      <c r="M51" s="24"/>
+      <c r="N51" s="24"/>
+      <c r="O51" s="24"/>
+      <c r="P51" s="24"/>
+    </row>
+    <row r="52" spans="2:16" ht="43.2">
+      <c r="I52" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="N52" s="21">
+        <f>MAX(N50,L51)</f>
+        <v>0.73775846532035805</v>
+      </c>
+      <c r="O52" s="19" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53" spans="2:16">
+      <c r="B53" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="23">
+        <v>7</v>
+      </c>
+      <c r="D53" s="27">
+        <v>0.36018</v>
+      </c>
+      <c r="E53" s="27">
+        <v>0.36068</v>
+      </c>
+      <c r="F53" s="27">
+        <v>0.36118</v>
+      </c>
+      <c r="G53" s="27">
+        <v>0.36168</v>
+      </c>
+      <c r="I53" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="J53" s="24">
+        <v>7</v>
+      </c>
+      <c r="K53" s="24"/>
+      <c r="L53" s="26">
+        <v>0.74717522483983601</v>
+      </c>
+      <c r="M53" s="24"/>
+      <c r="N53" s="24"/>
+      <c r="O53" s="24"/>
+      <c r="P53" s="24"/>
+    </row>
+    <row r="54" spans="2:16">
+      <c r="N54" s="21">
+        <f>MAX(N52,L53)</f>
+        <v>0.74717522483983601</v>
       </c>
     </row>
   </sheetData>
@@ -4164,7 +4548,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB787A30-BB0A-4678-A75A-EF41DE76C694}">
-  <dimension ref="B3:P40"/>
+  <dimension ref="B3:P44"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -5020,6 +5404,92 @@
         <v>1</v>
       </c>
     </row>
+    <row r="41" spans="2:16">
+      <c r="B41" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="23">
+        <v>6</v>
+      </c>
+      <c r="D41" s="27">
+        <v>0.99849900000000003</v>
+      </c>
+      <c r="E41" s="27">
+        <v>0.99899899999999997</v>
+      </c>
+      <c r="F41" s="27">
+        <v>0.99949900000000003</v>
+      </c>
+      <c r="G41" s="27">
+        <v>1</v>
+      </c>
+      <c r="I41" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="J41" s="24">
+        <v>6</v>
+      </c>
+      <c r="K41" s="24"/>
+      <c r="L41" s="26">
+        <v>8604.4979780305202</v>
+      </c>
+      <c r="M41" s="24"/>
+      <c r="N41" s="24"/>
+      <c r="O41" s="24"/>
+      <c r="P41" s="24"/>
+    </row>
+    <row r="42" spans="2:16" ht="28.8">
+      <c r="I42" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="N42" s="21">
+        <f>MAX(N40,L41)</f>
+        <v>8662.4825000000001</v>
+      </c>
+      <c r="O42" s="19" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16">
+      <c r="B43" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="23">
+        <v>7</v>
+      </c>
+      <c r="D43" s="27">
+        <v>1</v>
+      </c>
+      <c r="E43" s="27">
+        <v>0.4</v>
+      </c>
+      <c r="F43" s="27">
+        <v>1</v>
+      </c>
+      <c r="G43" s="27">
+        <v>1</v>
+      </c>
+      <c r="I43" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="J43" s="24">
+        <v>7</v>
+      </c>
+      <c r="K43" s="24"/>
+      <c r="L43" s="26">
+        <v>4540.3798008896001</v>
+      </c>
+      <c r="M43" s="24"/>
+      <c r="N43" s="24"/>
+      <c r="O43" s="24"/>
+      <c r="P43" s="24"/>
+    </row>
+    <row r="44" spans="2:16">
+      <c r="N44" s="21">
+        <f>MAX(N42,L43)</f>
+        <v>8662.4825000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B9:C28"/>
@@ -5037,7 +5507,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B451910E-E097-46FF-B069-9F3B8C7F2915}">
-  <dimension ref="B3:Q41"/>
+  <dimension ref="B3:Q45"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -5996,6 +6466,99 @@
         <v>1</v>
       </c>
     </row>
+    <row r="42" spans="2:17">
+      <c r="B42" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="23">
+        <v>6</v>
+      </c>
+      <c r="D42" s="27">
+        <v>0.45218000000000003</v>
+      </c>
+      <c r="E42" s="27">
+        <v>0.45258100000000001</v>
+      </c>
+      <c r="F42" s="27">
+        <v>0.45298100000000002</v>
+      </c>
+      <c r="G42" s="27">
+        <v>0.7</v>
+      </c>
+      <c r="H42" s="27">
+        <v>0.06</v>
+      </c>
+      <c r="J42" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="K42" s="24">
+        <v>6</v>
+      </c>
+      <c r="L42" s="24"/>
+      <c r="M42" s="26">
+        <v>-0.49607977761293698</v>
+      </c>
+      <c r="N42" s="24"/>
+      <c r="O42" s="24"/>
+      <c r="P42" s="24"/>
+      <c r="Q42" s="24"/>
+    </row>
+    <row r="43" spans="2:17" ht="43.2">
+      <c r="J43" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="O43" s="21">
+        <f>MAX(O41,M42)</f>
+        <v>-0.49607977761293698</v>
+      </c>
+      <c r="P43" s="19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="2:17">
+      <c r="B44" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="23">
+        <v>7</v>
+      </c>
+      <c r="D44" s="27">
+        <v>0.45218000000000003</v>
+      </c>
+      <c r="E44" s="27">
+        <v>0.45258100000000001</v>
+      </c>
+      <c r="F44" s="27">
+        <v>0.45298100000000002</v>
+      </c>
+      <c r="G44" s="27">
+        <v>0.7</v>
+      </c>
+      <c r="H44" s="27">
+        <v>0.06</v>
+      </c>
+      <c r="J44" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="K44" s="24">
+        <v>7</v>
+      </c>
+      <c r="L44" s="24"/>
+      <c r="M44" s="26">
+        <v>-0.39276604451561498</v>
+      </c>
+      <c r="N44" s="24"/>
+      <c r="O44" s="24"/>
+      <c r="P44" s="24"/>
+      <c r="Q44" s="24"/>
+    </row>
+    <row r="45" spans="2:17">
+      <c r="M45" s="20"/>
+      <c r="O45" s="21">
+        <f>MAX(O43,M44)</f>
+        <v>-0.39276604451561498</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B9:C28"/>
@@ -6013,7 +6576,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B58C19-2A2F-49AE-AB19-E8DF9CAE3947}">
-  <dimension ref="B3:R50"/>
+  <dimension ref="B3:R54"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -7245,6 +7808,12 @@
       <c r="K48" s="19" t="s">
         <v>76</v>
       </c>
+      <c r="L48" s="3">
+        <v>0.99</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="P48" s="21">
         <f>MAX(P46,N47)</f>
         <v>1.8037650755561301</v>
@@ -7300,6 +7869,12 @@
       <c r="K50" s="19" t="s">
         <v>84</v>
       </c>
+      <c r="L50" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="M50" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="P50" s="21">
         <f>MAX(P48,N49)</f>
         <v>1.8037650755561301</v>
@@ -7309,6 +7884,110 @@
       </c>
       <c r="R50" s="29" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="2:18">
+      <c r="B51" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="23">
+        <v>6</v>
+      </c>
+      <c r="D51" s="27">
+        <v>0.33411099999999999</v>
+      </c>
+      <c r="E51" s="27">
+        <v>0.33444400000000002</v>
+      </c>
+      <c r="F51" s="27">
+        <v>0.33477800000000002</v>
+      </c>
+      <c r="G51" s="27">
+        <v>0.33511099999999999</v>
+      </c>
+      <c r="H51" s="27">
+        <v>0.33544499999999999</v>
+      </c>
+      <c r="I51" s="27">
+        <v>0.68</v>
+      </c>
+      <c r="K51" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="L51" s="24">
+        <v>6</v>
+      </c>
+      <c r="M51" s="24"/>
+      <c r="N51" s="26">
+        <v>2.5841859527428799</v>
+      </c>
+      <c r="O51" s="24"/>
+      <c r="P51" s="24"/>
+      <c r="Q51" s="24"/>
+      <c r="R51" s="24"/>
+    </row>
+    <row r="52" spans="2:18" ht="43.2">
+      <c r="K52" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="L52" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="M52" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="P52" s="21">
+        <f>MAX(P50,N51)</f>
+        <v>2.5841859527428799</v>
+      </c>
+      <c r="Q52" s="19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="2:18">
+      <c r="B53" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="23">
+        <v>7</v>
+      </c>
+      <c r="D53" s="27">
+        <v>0.366122</v>
+      </c>
+      <c r="E53" s="27">
+        <v>0.36645499999999998</v>
+      </c>
+      <c r="F53" s="27">
+        <v>0.366788</v>
+      </c>
+      <c r="G53" s="27">
+        <v>0.367122</v>
+      </c>
+      <c r="H53" s="27">
+        <v>0.36745499999999998</v>
+      </c>
+      <c r="I53" s="27">
+        <v>0.68</v>
+      </c>
+      <c r="K53" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="L53" s="24">
+        <v>7</v>
+      </c>
+      <c r="M53" s="24"/>
+      <c r="N53" s="26">
+        <v>2.2258662517679002</v>
+      </c>
+      <c r="O53" s="24"/>
+      <c r="P53" s="24"/>
+      <c r="Q53" s="24"/>
+      <c r="R53" s="24"/>
+    </row>
+    <row r="54" spans="2:18">
+      <c r="P54" s="21">
+        <f>MAX(P52,N53)</f>
+        <v>2.5841859527428799</v>
       </c>
     </row>
   </sheetData>
@@ -7328,7 +8007,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0AA28BB-74D8-433B-A00A-14B553BBFF2F}">
-  <dimension ref="B3:T61"/>
+  <dimension ref="B3:T65"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.734375" customWidth="1"/>
@@ -9232,6 +9911,116 @@
         <v>1</v>
       </c>
     </row>
+    <row r="62" spans="2:20">
+      <c r="B62" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="23">
+        <v>6</v>
+      </c>
+      <c r="D62" s="27">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E62" s="27">
+        <v>4.6260999999999997E-2</v>
+      </c>
+      <c r="F62" s="27">
+        <v>0.1</v>
+      </c>
+      <c r="G62" s="27">
+        <v>0.1</v>
+      </c>
+      <c r="H62" s="27">
+        <v>4.7010999999999997E-2</v>
+      </c>
+      <c r="I62" s="27">
+        <v>4.7260999999999997E-2</v>
+      </c>
+      <c r="J62" s="27">
+        <v>4.7510999999999998E-2</v>
+      </c>
+      <c r="K62" s="27">
+        <v>4.7760999999999998E-2</v>
+      </c>
+      <c r="M62" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="N62" s="24">
+        <v>6</v>
+      </c>
+      <c r="O62" s="24"/>
+      <c r="P62" s="25">
+        <v>9.4167668191433993</v>
+      </c>
+      <c r="Q62" s="24"/>
+      <c r="R62" s="24"/>
+      <c r="S62" s="24"/>
+      <c r="T62" s="24"/>
+    </row>
+    <row r="63" spans="2:20" ht="57.6">
+      <c r="M63" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="R63" s="21">
+        <f>MAX(R61,P62)</f>
+        <v>9.6768866362245998</v>
+      </c>
+      <c r="S63" s="19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="64" spans="2:20">
+      <c r="B64" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="23">
+        <v>7</v>
+      </c>
+      <c r="D64" s="27">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E64" s="27">
+        <v>0.19</v>
+      </c>
+      <c r="F64" s="27">
+        <v>0</v>
+      </c>
+      <c r="G64" s="27">
+        <v>0</v>
+      </c>
+      <c r="H64" s="27">
+        <v>0.19</v>
+      </c>
+      <c r="I64" s="27">
+        <v>0.19</v>
+      </c>
+      <c r="J64" s="27">
+        <v>0.19</v>
+      </c>
+      <c r="K64" s="27">
+        <v>0.19</v>
+      </c>
+      <c r="M64" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="N64" s="24">
+        <v>7</v>
+      </c>
+      <c r="O64" s="24"/>
+      <c r="P64" s="25">
+        <v>9.6115899999999996</v>
+      </c>
+      <c r="Q64" s="24"/>
+      <c r="R64" s="24"/>
+      <c r="S64" s="24"/>
+      <c r="T64" s="24"/>
+    </row>
+    <row r="65" spans="18:18">
+      <c r="R65" s="21">
+        <f>MAX(R63,P64)</f>
+        <v>9.6768866362245998</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B9:C48"/>

</xml_diff>